<commit_message>
Remove obsolete JSON and text data files, and update the Excel conversion script and upload spreadsheets.
</commit_message>
<xml_diff>
--- a/1_Upload_Categories_Chirag.xlsx
+++ b/1_Upload_Categories_Chirag.xlsx
@@ -901,11 +901,7 @@
           <t>Chirag Singhal - MF FRONT LOADER 4700M CAB</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -955,11 +951,7 @@
           <t>Chirag Singhal - MF SMALL SQUARE BALERS</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1145,11 +1137,7 @@
           <t>Chirag Singhal - MF LARGE SQUARE BALERS</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1199,11 +1187,7 @@
           <t>Chirag Singhal - MF 3100 F ROUND BALERS</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1226,11 +1210,7 @@
           <t>Chirag Singhal - MF 3100 F PROTEC</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1253,11 +1233,7 @@
           <t>Chirag Singhal - MF 4100 V PROTEC</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -1307,11 +1283,7 @@
           <t>Chirag Singhal - MF 4100 V ROUND BALERS</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Level 2 Category</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>TRUE</t>

</xml_diff>